<commit_message>
complete bugs reports & other files
</commit_message>
<xml_diff>
--- a/QA/Test-Cases.xlsx
+++ b/QA/Test-Cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pro\source\repos\SauceDemo-Manual-Testing\QA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA73A63F-2256-4147-939F-B3D815CBCA48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEA9A8E8-7786-48EB-92CD-8E4ECC3D10AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="107">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -180,9 +180,6 @@
     <t>button to increase  quantity of product</t>
   </si>
   <si>
-    <t>user able to increase quantity</t>
-  </si>
-  <si>
     <t>user can't increase quantity</t>
   </si>
   <si>
@@ -327,9 +324,6 @@
     <t>sotoring in right way</t>
   </si>
   <si>
-    <t xml:space="preserve">user finish checkout and print </t>
-  </si>
-  <si>
     <t>finish don't work and user can't move on</t>
   </si>
   <si>
@@ -346,6 +340,15 @@
   </si>
   <si>
     <t>BUG-006</t>
+  </si>
+  <si>
+    <t>Performance</t>
+  </si>
+  <si>
+    <t>user can  increase quantity</t>
+  </si>
+  <si>
+    <t>user finish checkout and print invoice</t>
   </si>
 </sst>
 </file>
@@ -771,7 +774,7 @@
         <v>23</v>
       </c>
       <c r="J2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
@@ -803,7 +806,7 @@
         <v>24</v>
       </c>
       <c r="J3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
@@ -835,7 +838,7 @@
         <v>24</v>
       </c>
       <c r="J4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
@@ -859,13 +862,13 @@
         <v>21</v>
       </c>
       <c r="H5" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="I5" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="J5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
@@ -889,13 +892,13 @@
         <v>21</v>
       </c>
       <c r="H6" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="I6" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="J6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
@@ -912,26 +915,26 @@
         <v>47</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F7" s="2"/>
       <c r="G7" t="s">
-        <v>22</v>
+        <v>48</v>
       </c>
       <c r="H7" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="I7" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="I7" s="3" t="s">
-        <v>96</v>
-      </c>
       <c r="J7" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="K7" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="L7" s="3" t="s">
         <v>77</v>
-      </c>
-      <c r="L7" s="3" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.35">
@@ -942,7 +945,7 @@
         <v>34</v>
       </c>
       <c r="C8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D8" t="s">
         <v>16</v>
@@ -955,13 +958,13 @@
         <v>21</v>
       </c>
       <c r="H8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="I8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="J8" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
@@ -985,13 +988,13 @@
         <v>21</v>
       </c>
       <c r="H9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="J9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.35">
@@ -1015,19 +1018,19 @@
         <v>48</v>
       </c>
       <c r="H10" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="I10" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="I10" s="3" t="s">
-        <v>51</v>
-      </c>
       <c r="J10" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.35">
@@ -1038,43 +1041,43 @@
         <v>35</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>47</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F11" s="3"/>
       <c r="G11" s="3" t="s">
         <v>48</v>
       </c>
       <c r="H11" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="I11" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="I11" s="3" t="s">
+      <c r="J11" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="J11" s="3" t="s">
-        <v>77</v>
-      </c>
       <c r="K11" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C12" t="s">
         <v>53</v>
-      </c>
-      <c r="C12" t="s">
-        <v>54</v>
       </c>
       <c r="D12" t="s">
         <v>16</v>
@@ -1087,24 +1090,24 @@
         <v>22</v>
       </c>
       <c r="H12" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I12" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J12" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B13" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C13" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D13" t="s">
         <v>16</v>
@@ -1113,30 +1116,30 @@
         <v>44</v>
       </c>
       <c r="F13" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G13" t="s">
         <v>22</v>
       </c>
       <c r="H13" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I13" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J13" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C14" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D14" t="s">
         <v>16</v>
@@ -1145,30 +1148,30 @@
         <v>44</v>
       </c>
       <c r="F14" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G14" t="s">
         <v>22</v>
       </c>
       <c r="H14" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I14" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15" t="s">
         <v>52</v>
       </c>
-      <c r="B15" t="s">
-        <v>53</v>
-      </c>
       <c r="C15" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D15" t="s">
         <v>16</v>
@@ -1177,24 +1180,24 @@
         <v>44</v>
       </c>
       <c r="F15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G15" t="s">
         <v>22</v>
       </c>
       <c r="H15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J15" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B16" t="s">
         <v>42</v>
@@ -1213,13 +1216,13 @@
         <v>45</v>
       </c>
       <c r="H16" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I16" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="J16" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.35">
@@ -1230,7 +1233,7 @@
         <v>34</v>
       </c>
       <c r="C17" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D17" t="s">
         <v>16</v>
@@ -1243,13 +1246,13 @@
         <v>45</v>
       </c>
       <c r="H17" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I17" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J17" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.35">
@@ -1260,7 +1263,7 @@
         <v>34</v>
       </c>
       <c r="C18" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D18" t="s">
         <v>16</v>
@@ -1273,121 +1276,121 @@
         <v>45</v>
       </c>
       <c r="H18" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="I18" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J18" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>47</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F19" s="2"/>
       <c r="G19" s="3" t="s">
         <v>48</v>
       </c>
       <c r="H19" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="I19" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="I19" s="3" t="s">
-        <v>83</v>
-      </c>
       <c r="J19" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>47</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F20" s="2"/>
       <c r="G20" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>34</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D21" s="3" t="s">
         <v>47</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F21" s="2"/>
       <c r="G21" s="3" t="s">
-        <v>70</v>
+        <v>104</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>

</xml_diff>